<commit_message>
remove flowdir2 from test data
doesn't parse correctly due to issue in FCSFiles.jl
</commit_message>
<xml_diff>
--- a/test/inputs/flowdir.xlsx
+++ b/test/inputs/flowdir.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53D97219-15D7-6641-BFC2-4D9075BB9202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350F790F-843F-5447-A066-6181C4D2563D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19420" yWindow="7480" windowWidth="18980" windowHeight="9440" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
   <si>
     <t>Plate</t>
   </si>
@@ -91,9 +91,6 @@
   </si>
   <si>
     <t>a5</t>
-  </si>
-  <si>
-    <t>$GITHUB_WORKSPACE/test/inputs/flowdir2</t>
   </si>
   <si>
     <t>$GITHUB_WORKSPACE/test/inputs/small.fcs</t>
@@ -479,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2569E313-B3CC-438F-A253-EA0F3E8D819B}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -527,7 +524,7 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -541,24 +538,13 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4">
         <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added flowdir2 to test
include testing for alternate naming schemes (A01 rather than A1)
</commit_message>
<xml_diff>
--- a/test/inputs/flowdir.xlsx
+++ b/test/inputs/flowdir.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350F790F-843F-5447-A066-6181C4D2563D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1382E6AB-93FA-4044-8780-AA553813A089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19420" yWindow="7480" windowWidth="18980" windowHeight="9440" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <si>
     <t>Plate</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>$GITHUB_WORKSPACE/test/inputs/biotek-data.csv</t>
+  </si>
+  <si>
+    <t>$GITHUB_WORKSPACE/test/inputs/flowdir2</t>
   </si>
 </sst>
 </file>
@@ -476,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2569E313-B3CC-438F-A253-EA0F3E8D819B}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -545,6 +548,18 @@
       </c>
       <c r="E4">
         <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="E5">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>